<commit_message>
Report how much the uncast scan actually covered
Counts companies reached, season pages read and production pages opened,
and prints them at the end, so a run states its own coverage instead of
leaving it to be guessed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/uncast_roles.xlsx
+++ b/uncast_roles.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uncast roles" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Uncast roles'!$A$1:$L$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Uncast roles'!$A$1:$L$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -559,7 +559,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nationaltheater Mannheim</t>
+          <t>Bayerische Staatsoper</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -569,33 +569,33 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Der Ring an einem Abend</t>
+          <t>DIE KAMELIENDAME</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Grimgerde</t>
+          <t>Manon Lescaut</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Dramatischer Mezzosopran</t>
+          <t>Jugendlich-dramatischer Sopran</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Mezzo</t>
+          <t>Soprano</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Die Walkuere</t>
+          <t>Manon Lescaut</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Wagner</t>
+          <t>Puccini</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>http://www.nationaltheater-mannheim.de/spielplan/a-z/der-ring-an-einem-abend/</t>
+          <t>https://www.staatsoper.de/stuecke/die-kameliendame</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Semperoper Dresden</t>
+          <t>Bayerische Staatsoper</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -627,17 +627,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Don Carlo</t>
+          <t>DIE KAMELIENDAME</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Il Conte di Lerma</t>
+          <t>Des Grieux</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Charaktertenor</t>
+          <t>Jugendlicher Heldentenor</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -648,12 +648,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Don Carlo</t>
+          <t>Manon Lescaut</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Verdi</t>
+          <t>Puccini</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://www.semperoper.de/spielplan/stuecke/stid/don-carlo/61447.html</t>
+          <t>https://www.staatsoper.de/stuecke/die-kameliendame</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -675,7 +675,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Semperoper Dresden</t>
+          <t>Bayerische Staatsoper</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -685,33 +685,33 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Don Carlo</t>
+          <t>DIE KAMELIENDAME</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Un Frate</t>
+          <t>Olympia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Serioeser Bass</t>
+          <t>Koloratursopran</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Bass</t>
+          <t>Soprano</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Don Carlo</t>
+          <t>Les contes d'Hoffmann</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Verdi</t>
+          <t>Offenbach</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.semperoper.de/spielplan/stuecke/stid/don-carlo/61447.html</t>
+          <t>https://www.staatsoper.de/stuecke/die-kameliendame</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -733,7 +733,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Semperoper Dresden</t>
+          <t>Deutsche Oper am Rhein</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -743,33 +743,33 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>La bohème</t>
+          <t>Il barbiere di Siviglia</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Musetta</t>
+          <t>Bartolo</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lyrischer Sopran / Soubrette</t>
+          <t>Spielbass</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Soprano</t>
+          <t>Bass</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>La boheme</t>
+          <t>Le nozze di Figaro</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Puccini</t>
+          <t>Mozart</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.semperoper.de/spielplan/stuecke/stid/boheme/147.html</t>
+          <t>https://operamrhein.de/spielplan/produktionen/il-barbiere-di-siviglia/</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -801,33 +801,33 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>La bohème</t>
+          <t>Don Carlo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colline</t>
+          <t>Il Conte di Lerma</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Serioeser Bass</t>
+          <t>Charaktertenor</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bass</t>
+          <t>Tenor</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>La boheme</t>
+          <t>Don Carlo</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Puccini</t>
+          <t>Verdi</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.semperoper.de/spielplan/stuecke/stid/boheme/147.html</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/don-carlo/61447.html</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -849,53 +849,53 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nederlandse Reisopera</t>
+          <t>Semperoper Dresden</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Impressions de Pelléas</t>
+          <t>Don Carlo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Yniold</t>
+          <t>Un Frate</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Soubrette / Knabensopran</t>
+          <t>Serioeser Bass</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Soprano</t>
+          <t>Bass</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Pelleas et Melisande</t>
+          <t>Don Carlo</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Debussy</t>
+          <t>Verdi</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>NN</t>
+          <t>N.N.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.reisopera.nl/programma/impressions-de-pelleas</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/don-carlo/61447.html</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -907,43 +907,43 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Oper Graz</t>
+          <t>Semperoper Dresden</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kalender</t>
+          <t>La bohème</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Der Pfleger des Orest | Ein alter Diener</t>
+          <t>Musetta</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Lyrischer Sopran / Soubrette</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Soprano</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>La boheme</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Puccini</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.oper-graz.com/spielplan/kalender/</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/boheme/147.html</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -965,53 +965,53 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Opera de Lyon</t>
+          <t>Semperoper Dresden</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nuit de mai</t>
+          <t>La bohème</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>La Marâtre</t>
+          <t>Colline</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Serioeser Bass</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Bass</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>La boheme</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Puccini</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>NN</t>
+          <t>N.N.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.opera-lyon.com/fr/programmation/saison-2026-2027/opera/nuit-de-mai</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/boheme/147.html</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1023,53 +1023,53 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Opera de Lyon</t>
+          <t>Semperoper Dresden</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Leïla Martial &amp; Elie Dufour "Karma Bazar"</t>
+          <t>Die Zauberflöte</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>– son,</t>
+          <t>Papagena</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Soubrette</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Soprano</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Die Zauberfloete</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Mozart</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>NN</t>
+          <t>N.N.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.opera-lyon.com/fr/programmation/saison-2026-2027/opera-underground/leila-martial-elie-dufour-karma-bazar</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/zauberfloete/61859.html</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1081,53 +1081,53 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Theatre des Champs-Elysees</t>
+          <t>Semperoper Dresden</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hippolyte et Aricie</t>
+          <t>Die Zauberflöte</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>| L'Amour / Une Matelote / Une Bergère / Une Prêtresse</t>
+          <t>Sarastro</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Serioeser Bass</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Bass</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Die Zauberfloete</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Mozart</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>NN</t>
+          <t>N.N.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.theatrechampselysees.fr/saison-2026-27/opera-en-concert/hippolyte-et-aricie</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/zauberfloete/61859.html</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1139,7 +1139,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Oper Stuttgart</t>
+          <t>Semperoper Dresden</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1149,33 +1149,33 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Atatürk</t>
+          <t>Die Zauberflöte</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Enver Pascha/ 5. Frau, die Überassimilierte</t>
+          <t>Tamino</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Lyrischer Tenor</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Tenor</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Die Zauberfloete</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Mozart</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.staatsoper-stuttgart.de/spielplan/a-z/atatuerk/</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/zauberfloete/61859.html</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1197,53 +1197,53 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Folkoperan</t>
+          <t>Semperoper Dresden</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Olympiaden</t>
+          <t>Die Zauberflöte</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Prins av Kreta, besluten att vinna Olympiaden och prinsessan Aristeas hand.</t>
+          <t>Sprecher</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Bass-Bariton</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Bass-baritone</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Die Zauberfloete</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>N.A.</t>
+          <t>Mozart</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Nn</t>
+          <t>N.N.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://folkoperan.se/uppsattningar/olympiaden/</t>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/zauberfloete/61859.html</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1252,8 +1252,1578 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Semperoper Dresden</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Die Zauberflöte</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Papageno</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Kavalierbariton</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Lyrischer Bariton / Spielbariton</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Baritone</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Die Zauberfloete</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Mozart</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/zauberfloete/61859.html</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Semperoper Dresden</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Die Zauberflöte</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Pamina</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Lyrischer Sopran</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Soprano</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Die Zauberfloete</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Mozart</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://www.semperoper.de/spielplan/stuecke/stid/zauberfloete/61859.html</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Theater Dortmund</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Das Geheimnis der Knusperhexe</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sandmännchen</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Soubrette</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Soprano</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Haensel und Gretel</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Humperdinck</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://www.theaterdo.de/produktionen/detail/das-geheimnis-der-knusperhexe/</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Opera North</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Audio Described Performances</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Rigoletto</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Charakterbariton / Verdi-Bariton</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Baritone</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Rigoletto</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Verdi</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://www.operanorth.co.uk/access/audio-described-performances/</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Opera North</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Audio Described Performances</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Don Giovanni</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Kavalierbariton</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Baritone</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Don Giovanni</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Mozart</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://www.operanorth.co.uk/access/audio-described-performances/</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Oper Graz</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Kalender</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Der Pfleger des Orest | Ein alter Diener</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://www.oper-graz.com/spielplan/kalender/</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Pacific Opera Victoria</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Hansel &amp; Gretel</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Sandman/Dew Fairy</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://pacificopera.ca/event/hansel-gretel/</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Opera Comique</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>L'équipe de l'Opéra-Comique</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Adjointe à la DRH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://www.opera-comique.com/en/node/1655</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Opera Comique</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>L'équipe de l'Opéra-Comique</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Adjointe paie, responsable du SIRH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://www.opera-comique.com/en/node/1655</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Opera de Lyon</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Nuit de mai</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>La Marâtre</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://www.opera-lyon.com/fr/programmation/saison-2026-2027/opera/nuit-de-mai</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Opera de Lyon</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Leïla Martial &amp; Elie Dufour "Karma Bazar"</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>– son,</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://www.opera-lyon.com/fr/programmation/saison-2026-2027/opera-underground/leila-martial-elie-dufour-karma-bazar</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Deutsche Oper Berlin</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>In 80 Tagen um die Welt</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Schaffner / Sailor / Häuptling der Apachen</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>N. N.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://www.deutscheoperberlin.de/de_DE/production/in-80-tagen-um-die-welt.1385725</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Deutsche Oper Berlin</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Le nozze di Figaro</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>N. N.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>N. N.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://www.deutscheoperberlin.de/de_DE/production/le-nozze-di-figaro.1385793</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Oldenburgisches Staatstheater</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>4. Sinfoniekonzert</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Solist:innen</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>N. N.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://www.staatstheater.de/programm/konzert/sinfoniekonzerte/spielzeit-2627/4-sinfoniekonzert</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Oldenburgisches Staatstheater</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>The Sound of Music</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Louisa, 13 Jahre</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://www.staatstheater.de/programm/musiktheater/spielzeit-2627/the-sound-of-music</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Oldenburgisches Staatstheater</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>The Sound of Music</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Kurt, 10 Jahre</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://www.staatstheater.de/programm/musiktheater/spielzeit-2627/the-sound-of-music</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Oldenburgisches Staatstheater</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>The Sound of Music</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Brigitta, 9 Jahre</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://www.staatstheater.de/programm/musiktheater/spielzeit-2627/the-sound-of-music</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Oldenburgisches Staatstheater</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>The Sound of Music</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Marta, 7 Jahre</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://www.staatstheater.de/programm/musiktheater/spielzeit-2627/the-sound-of-music</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Oldenburgisches Staatstheater</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>The Sound of Music</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Gretl, die Jüngste</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://www.staatstheater.de/programm/musiktheater/spielzeit-2627/the-sound-of-music</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Oper Stuttgart</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Atatürk</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Enver Pascha/ 5. Frau, die Überassimilierte</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://www.staatsoper-stuttgart.de/spielplan/a-z/atatuerk/</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Theater Bonn</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Der Barbier von Sevilla</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Tanz - Swing</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://www.theater-bonn.de/de/programm/der-barbier-von-sevilla/227939</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Welcome to Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>“Drinking tea in various attitudes of deep abstraction”</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>tbc</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://bamptonopera.org/operadetail.htm?event=52</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Welcome to Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Fidelity and fishing: La vera costanza</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>tbc</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://bamptonopera.org/operadetail.htm?event=63</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Welcome to Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>‘Sir John in Love’</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>tbc</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://bamptonopera.org/operadetail.htm?event=62</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Welcome to Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>The Merry Wives of Windsor: operatic and music theatre settings</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>tbc</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://bamptonopera.org/operadetail.htm?event=62</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Welcome to Bampton Classical Opera</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Waiting for Figaro - two abandoned operas and a singspiel</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>tbc</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://bamptonopera.org/operadetail.htm?event=66</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Opera North</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Audio Described Performances</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>N.A.</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://www.operanorth.co.uk/access/audio-described-performances/</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L14"/>
+  <autoFilter ref="A1:L41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>